<commit_message>
trying enqCNAS and fixing date
</commit_message>
<xml_diff>
--- a/new_EnquetCNAS.xlsx
+++ b/new_EnquetCNAS.xlsx
@@ -387,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -438,31 +438,31 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="str">
-        <v>3988</v>
+        <v>119</v>
       </c>
       <c r="C2" s="2" t="str">
         <v/>
       </c>
       <c r="D2" s="2" t="str">
-        <v>HMIDI</v>
+        <v>BELABBAS</v>
       </c>
       <c r="E2" s="2" t="str">
-        <v>ALI</v>
+        <v>ABDELKADER</v>
       </c>
       <c r="F2" s="2" t="str">
-        <v>31/12/1974</v>
+        <v>21/02/1970</v>
       </c>
       <c r="G2" s="2" t="str">
-        <v xml:space="preserve"> 245  03    </v>
+        <v/>
       </c>
       <c r="H2" s="2" t="str">
-        <v>426</v>
+        <v>405</v>
       </c>
       <c r="I2" s="2" t="str">
-        <v>MOHAMMED</v>
+        <v>ABDELHAFID</v>
       </c>
       <c r="J2" s="2" t="str">
-        <v>AMOURIA GHARSA</v>
+        <v>BELABBAS FATIMA</v>
       </c>
       <c r="K2" s="2" t="str">
         <v>M</v>
@@ -471,10 +471,10 @@
         <v/>
       </c>
       <c r="M2" s="2" t="str">
-        <v>BESBAS</v>
+        <v>TOUGGOURT</v>
       </c>
       <c r="N2" s="2" t="str">
-        <v>Ouled Djellal</v>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -482,31 +482,31 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="str">
-        <v>5158</v>
+        <v>1219</v>
       </c>
       <c r="C3" s="2" t="str">
         <v/>
       </c>
       <c r="D3" s="2" t="str">
-        <v>BELKEMARI</v>
+        <v>TABOUN</v>
       </c>
       <c r="E3" s="2" t="str">
-        <v>ALI</v>
+        <v>YOUCEF</v>
       </c>
       <c r="F3" s="2" t="str">
-        <v>03/03/1991</v>
+        <v>17/08/1976</v>
       </c>
       <c r="G3" s="2" t="str">
-        <v xml:space="preserve">  01   </v>
+        <v/>
       </c>
       <c r="H3" s="2" t="str">
-        <v>53</v>
+        <v>1554</v>
       </c>
       <c r="I3" s="2" t="str">
-        <v>LAHADJ</v>
+        <v>DAHMANE</v>
       </c>
       <c r="J3" s="2" t="str">
-        <v>BELKEMARI RAISSA</v>
+        <v>BOUTADJINE MESSAOUDA</v>
       </c>
       <c r="K3" s="2" t="str">
         <v>M</v>
@@ -518,7 +518,7 @@
         <v>TOUGGOURT</v>
       </c>
       <c r="N3" s="2" t="str">
-        <v>Touggourt</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -526,34 +526,34 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="str">
-        <v>3884</v>
+        <v>1219</v>
       </c>
       <c r="C4" s="2" t="str">
         <v/>
       </c>
       <c r="D4" s="2" t="str">
-        <v>GHIABA</v>
+        <v>TABOUN</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v>KAMAL</v>
+        <v xml:space="preserve">MERIEM </v>
       </c>
       <c r="F4" s="2" t="str">
-        <v>21/02/1985</v>
+        <v>31/12/1985</v>
       </c>
       <c r="G4" s="2" t="str">
-        <v xml:space="preserve"> 664  06   01  </v>
+        <v/>
       </c>
       <c r="H4" s="2" t="str">
-        <v>138</v>
+        <v/>
       </c>
       <c r="I4" s="2" t="str">
-        <v>SAAD</v>
+        <v>MOHAMMED</v>
       </c>
       <c r="J4" s="2" t="str">
-        <v>GHIABA AICHA</v>
+        <v>BENNADJI FATNA</v>
       </c>
       <c r="K4" s="2" t="str">
-        <v>M</v>
+        <v>F</v>
       </c>
       <c r="L4" s="2" t="str">
         <v/>
@@ -562,232 +562,12 @@
         <v>TOUGGOURT</v>
       </c>
       <c r="N4" s="2" t="str">
-        <v>Touggourt</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>3670</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D5" s="2" t="str">
-        <v>DEBBAGH</v>
-      </c>
-      <c r="E5" s="2" t="str">
-        <v>ABDELDJALIL</v>
-      </c>
-      <c r="F5" s="2" t="str">
-        <v>23/05/1986</v>
-      </c>
-      <c r="G5" s="2" t="str">
-        <v xml:space="preserve"> 01   04  </v>
-      </c>
-      <c r="H5" s="2" t="str">
-        <v>260</v>
-      </c>
-      <c r="I5" s="2" t="str">
-        <v>ALI</v>
-      </c>
-      <c r="J5" s="2" t="str">
-        <v>BEN GAG RACHIDA</v>
-      </c>
-      <c r="K5" s="2" t="str">
-        <v>M</v>
-      </c>
-      <c r="L5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M5" s="2" t="str">
-        <v>TOUGGOURT</v>
-      </c>
-      <c r="N5" s="2" t="str">
-        <v>Touggourt</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>3380</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D6" s="2" t="str">
-        <v>KHELAFI</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>YASMINA</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>16/12/1974</v>
-      </c>
-      <c r="G6" s="2" t="str">
-        <v xml:space="preserve">    21  03 </v>
-      </c>
-      <c r="H6" s="2" t="str">
-        <v>3861</v>
-      </c>
-      <c r="I6" s="2" t="str">
-        <v>MOHAMMED</v>
-      </c>
-      <c r="J6" s="2" t="str">
-        <v>KHELAFI SALIHA</v>
-      </c>
-      <c r="K6" s="2" t="str">
-        <v>F</v>
-      </c>
-      <c r="L6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M6" s="2" t="str">
-        <v>BISKRA</v>
-      </c>
-      <c r="N6" s="2" t="str">
-        <v>Biskra</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>2340</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D7" s="2" t="str">
-        <v>MECHICHE</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>HAMZA</v>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v>02/10/1985</v>
-      </c>
-      <c r="G7" s="2" t="str">
-        <v xml:space="preserve">     21  03 </v>
-      </c>
-      <c r="H7" s="2" t="str">
-        <v>618</v>
-      </c>
-      <c r="I7" s="2" t="str">
-        <v>LAKHDAR</v>
-      </c>
-      <c r="J7" s="2" t="str">
-        <v>BOUGHERARA FATMA</v>
-      </c>
-      <c r="K7" s="2" t="str">
-        <v>M</v>
-      </c>
-      <c r="L7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M7" s="2" t="str">
-        <v>TOUGGOURT</v>
-      </c>
-      <c r="N7" s="2" t="str">
-        <v>Touggourt</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="str">
-        <v>5168</v>
-      </c>
-      <c r="C8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D8" s="2" t="str">
-        <v>KEMARI</v>
-      </c>
-      <c r="E8" s="2" t="str">
-        <v>AMOR</v>
-      </c>
-      <c r="F8" s="2" t="str">
-        <v>11/08/1987</v>
-      </c>
-      <c r="G8" s="2" t="str">
-        <v xml:space="preserve">   </v>
-      </c>
-      <c r="H8" s="2" t="str">
-        <v>382</v>
-      </c>
-      <c r="I8" s="2" t="str">
-        <v>LABIDI</v>
-      </c>
-      <c r="J8" s="2" t="str">
-        <v>KEMARI MERIEM</v>
-      </c>
-      <c r="K8" s="2" t="str">
-        <v>M</v>
-      </c>
-      <c r="L8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M8" s="2" t="str">
-        <v>TOUGGOURT</v>
-      </c>
-      <c r="N8" s="2" t="str">
-        <v>Touggourt</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="str">
-        <v>1875</v>
-      </c>
-      <c r="C9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D9" s="2" t="str">
-        <v>TOUMI</v>
-      </c>
-      <c r="E9" s="2" t="str">
-        <v>MOHAMMED</v>
-      </c>
-      <c r="F9" s="2" t="str">
-        <v>31/12/1970</v>
-      </c>
-      <c r="G9" s="2" t="str">
-        <v xml:space="preserve">  02  2  199 </v>
-      </c>
-      <c r="H9" s="2" t="str">
-        <v>472</v>
-      </c>
-      <c r="I9" s="2" t="str">
-        <v>MOKHTAR</v>
-      </c>
-      <c r="J9" s="2" t="str">
-        <v>TOUMI SAIDA</v>
-      </c>
-      <c r="K9" s="2" t="str">
-        <v>M</v>
-      </c>
-      <c r="L9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M9" s="2" t="str">
-        <v>SELMANA</v>
-      </c>
-      <c r="N9" s="2" t="str">
-        <v>Djelfa</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>